<commit_message>
WIP: snapshot cantieri (excel monitor in ricalcolo, dossier prop in lavorazione)
</commit_message>
<xml_diff>
--- a/report/MONITOR_CHALLENGE.xlsx
+++ b/report/MONITOR_CHALLENGE.xlsx
@@ -9492,7 +9492,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:K251">
+  <conditionalFormatting sqref="K2:K251">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$K2="VIOLAZIONE"</formula>
     </cfRule>
@@ -10449,7 +10449,7 @@
         </is>
       </c>
       <c r="B4" s="26">
-        <f>IFERROR(LOOKUP(2,1/(GIORNALIERO!B2:B251&lt;&gt;""),GIORNALIERO!B2:B251),IMPOSTAZIONI!B3)</f>
+        <f>IFERROR(INDEX(GIORNALIERO!B2:B251,COUNT(GIORNALIERO!$B$2:$B$251)),IMPOSTAZIONI!B3)</f>
         <v/>
       </c>
       <c r="C4" s="25" t="inlineStr">
@@ -10465,7 +10465,7 @@
         </is>
       </c>
       <c r="B5" s="26">
-        <f>IFERROR(LOOKUP(2,1/(GIORNALIERO!B2:B251&lt;&gt;""),GIORNALIERO!B2:B251),IMPOSTAZIONI!B3)+SUM(PRELIEVI!B2:B61)-IMPOSTAZIONI!B3</f>
+        <f>IFERROR(INDEX(GIORNALIERO!B2:B251,COUNT(GIORNALIERO!$B$2:$B$251)),IMPOSTAZIONI!B3)+SUM(PRELIEVI!B2:B61)-IMPOSTAZIONI!B3</f>
         <v/>
       </c>
       <c r="C5" s="25" t="inlineStr"/>
@@ -10538,7 +10538,7 @@
         </is>
       </c>
       <c r="B11" s="26">
-        <f>IFERROR(LOOKUP(2,1/(GIORNALIERO!B2:B251&lt;&gt;""),GIORNALIERO!B2:B251),IMPOSTAZIONI!B3)-IMPOSTAZIONI!B3</f>
+        <f>IFERROR(INDEX(GIORNALIERO!B2:B251,COUNT(GIORNALIERO!$B$2:$B$251)),IMPOSTAZIONI!B3)-IMPOSTAZIONI!B3</f>
         <v/>
       </c>
       <c r="C11" s="25" t="inlineStr">
@@ -10554,7 +10554,7 @@
         </is>
       </c>
       <c r="B12" s="26">
-        <f>IFERROR(LOOKUP(2,1/(GIORNALIERO!B2:B251&lt;&gt;""),GIORNALIERO!B2:B251),IMPOSTAZIONI!B3)-IMPOSTAZIONI!B10</f>
+        <f>IFERROR(INDEX(GIORNALIERO!B2:B251,COUNT(GIORNALIERO!$B$2:$B$251)),IMPOSTAZIONI!B3)-IMPOSTAZIONI!B10</f>
         <v/>
       </c>
       <c r="C12" s="25" t="inlineStr">

</xml_diff>